<commit_message>
Finalize QA evidence, private data provenance, and branch setup guide
</commit_message>
<xml_diff>
--- a/qa/Ankit_Karki_QA_Workbook.xlsx
+++ b/qa/Ankit_Karki_QA_Workbook.xlsx
@@ -22,7 +22,7 @@
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Fixture_3!$A$1:$L$61</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Fixture_4!$A$1:$L$61</definedName>
     <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">Fixture_5!$A$1:$L$61</definedName>
-    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Issue_Log!$A$1:$H$15</definedName>
+    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Issue_Log!$A$1:$H$16</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="178">
   <si>
     <t xml:space="preserve">ANKIT KARKI | INDEPENDENT QA</t>
   </si>
@@ -342,7 +342,7 @@
     <t xml:space="preserve">Use fixed AvgCH AvgCD AvgCA triplet and valid common sample</t>
   </si>
   <si>
-    <t xml:space="preserve">Design corrected; verify runtime</t>
+    <t xml:space="preserve">Verified fixed AvgC runtime benchmark</t>
   </si>
   <si>
     <t xml:space="preserve">Ankit Karki</t>
@@ -360,7 +360,7 @@
     <t xml:space="preserve">Expand grid until omitted mass below 1e-8 and record tail</t>
   </si>
   <si>
-    <t xml:space="preserve">Design corrected; verify tests</t>
+    <t xml:space="preserve">Verified adaptive tail tests and actual run</t>
   </si>
   <si>
     <t xml:space="preserve">Proposal mathematical approach</t>
@@ -375,7 +375,7 @@
     <t xml:space="preserve">Use first complete date boundary at or after 190 results</t>
   </si>
   <si>
-    <t xml:space="preserve">Design corrected; verify output</t>
+    <t xml:space="preserve">Verified Jan 1 complete-date boundary</t>
   </si>
   <si>
     <t xml:space="preserve">Proposal season backtest</t>
@@ -393,6 +393,9 @@
     <t xml:space="preserve">Skip full warmup date and report actual evaluated count</t>
   </si>
   <si>
+    <t xml:space="preserve">Verified 280 eligible rows for this snapshot</t>
+  </si>
+  <si>
     <t xml:space="preserve">Proposal walk-forward protocol</t>
   </si>
   <si>
@@ -456,7 +459,7 @@
     <t xml:space="preserve">Obtain authoritative 2025/26 table and reconcile numbers</t>
   </si>
   <si>
-    <t xml:space="preserve">Pending manual verification</t>
+    <t xml:space="preserve">Partial independent comparison; official full table still pending</t>
   </si>
   <si>
     <t xml:space="preserve">QA case D06</t>
@@ -504,7 +507,7 @@
     <t xml:space="preserve">Ignore raw CSVs in public Git; use private coursework copies and attribution</t>
   </si>
   <si>
-    <t xml:space="preserve">Implemented locally; verify before push</t>
+    <t xml:space="preserve">Verified raw CSVs ignored before public branch push</t>
   </si>
   <si>
     <t xml:space="preserve">QA-012</t>
@@ -543,10 +546,28 @@
     <t xml:space="preserve">Replace workbook grid formulas with direct EXP powers FACT Poisson definition and recalculate</t>
   </si>
   <si>
-    <t xml:space="preserve">Fix applied; re-verification pending</t>
+    <t xml:space="preserve">Resolved; zero formula errors and all five rate checks agree</t>
   </si>
   <si>
     <t xml:space="preserve">scripts/build_qa_workbook.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QA-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coding worker unexpectedly pushed partial live refinement to main instead of leaving local changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restored original main contents with regular revert 6d621c7; complete project isolated on review branch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolved; verify original main diff empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Git main repair commit 6d621c7</t>
   </si>
 </sst>
 </file>
@@ -8391,7 +8412,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8524,18 +8545,18 @@
         <v>118</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>103</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>98</v>
@@ -8544,24 +8565,24 @@
         <v>116</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>103</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>98</v>
@@ -8570,24 +8591,24 @@
         <v>99</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>98</v>
@@ -8596,24 +8617,24 @@
         <v>99</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>98</v>
@@ -8622,50 +8643,50 @@
         <v>116</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>103</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>98</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>98</v>
@@ -8674,24 +8695,24 @@
         <v>116</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>98</v>
@@ -8700,16 +8721,16 @@
         <v>116</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>104</v>
@@ -8717,33 +8738,33 @@
     </row>
     <row r="13" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>98</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>98</v>
@@ -8752,24 +8773,24 @@
         <v>116</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>103</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>98</v>
@@ -8778,23 +8799,49 @@
         <v>116</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>103</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:H16"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>